<commit_message>
flow des resultats vserion 1
</commit_message>
<xml_diff>
--- a/public/modele_listes.xlsx
+++ b/public/modele_listes.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa5cdb37f8cded9e/CAMPS^M/A/Emploi/CNX 4.0/CNX/Clients/SEEG/Elections professionnelles/Modèles importation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F44CB667-4F3A-4AC6-B307-D2F14471A915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{F44CB667-4F3A-4AC6-B307-D2F14471A915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64D0D79A-93DD-4DAA-AD6A-04214D4D6FE1}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04DB11DA-5E37-4FEB-B856-E7AD3B9D565E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{04DB11DA-5E37-4FEB-B856-E7AD3B9D565E}"/>
   </bookViews>
   <sheets>
     <sheet name="Listes" sheetId="1" r:id="rId1"/>
+    <sheet name="Exemple_Listes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="25">
   <si>
     <t>Genre_Suppleant</t>
   </si>
@@ -66,13 +67,61 @@
   </si>
   <si>
     <t>Acronyme_Representation</t>
+  </si>
+  <si>
+    <t>Encadrement</t>
+  </si>
+  <si>
+    <t>Femme</t>
+  </si>
+  <si>
+    <t>Homme</t>
+  </si>
+  <si>
+    <t>Exécution</t>
+  </si>
+  <si>
+    <t>Syndicat A</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>SB</t>
+  </si>
+  <si>
+    <t>Syndicat B</t>
+  </si>
+  <si>
+    <t>Etablissement E</t>
+  </si>
+  <si>
+    <t>Nom et prénom</t>
+  </si>
+  <si>
+    <t>Nom et prénom Suppléant</t>
+  </si>
+  <si>
+    <t>Matricule_Titulaire</t>
+  </si>
+  <si>
+    <t>Age_Titulaire</t>
+  </si>
+  <si>
+    <t>Matricule_Suppleant</t>
+  </si>
+  <si>
+    <t>Age_Suppleant</t>
+  </si>
+  <si>
+    <t>Ancienneté_Suppleant</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -83,6 +132,19 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="0" tint="-0.249977111117893"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0" tint="-0.249977111117893"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -124,10 +186,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -143,6 +209,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -470,21 +540,21 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.19921875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.69921875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.69921875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="21.5" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="11.19921875" style="1"/>
+    <col min="4" max="5" width="14.69921875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="21.5" style="1" customWidth="1"/>
+    <col min="11" max="11" width="22.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="11.19921875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -498,22 +568,900 @@
         <v>5</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>0</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0E9AB15-CA87-404F-86A7-AF364CDE7DEB}">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="A1:N169"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.8984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="44.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.8984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="44.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.09765625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="62.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="22" style="1" customWidth="1"/>
+    <col min="9" max="10" width="23.19921875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="55.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="11.19921875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1000</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="6">
+        <v>35</v>
+      </c>
+      <c r="I2" s="5">
+        <v>5</v>
+      </c>
+      <c r="J2" s="5">
+        <v>2000</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="4">
+        <v>45</v>
+      </c>
+      <c r="N2" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1001</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="6">
+        <v>46</v>
+      </c>
+      <c r="I3" s="5">
+        <v>7</v>
+      </c>
+      <c r="J3" s="5">
+        <v>2001</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M3" s="4">
+        <v>46</v>
+      </c>
+      <c r="N3" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="4">
+        <v>1002</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="6">
+        <v>44</v>
+      </c>
+      <c r="I4" s="5">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5">
+        <v>2002</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4" s="4">
+        <v>47</v>
+      </c>
+      <c r="N4" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+    </row>
+    <row r="17" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+    </row>
+    <row r="19" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="22" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+    </row>
+    <row r="27" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+    </row>
+    <row r="28" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+    </row>
+    <row r="29" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+    </row>
+    <row r="33" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+    </row>
+    <row r="34" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+    </row>
+    <row r="35" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+    </row>
+    <row r="36" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+    </row>
+    <row r="37" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+    </row>
+    <row r="38" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+    </row>
+    <row r="39" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+    </row>
+    <row r="40" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+    </row>
+    <row r="41" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+    </row>
+    <row r="42" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+    </row>
+    <row r="43" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+    </row>
+    <row r="44" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+    </row>
+    <row r="45" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+    </row>
+    <row r="46" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+    </row>
+    <row r="47" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+    </row>
+    <row r="48" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+    </row>
+    <row r="49" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+    </row>
+    <row r="50" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+    </row>
+    <row r="51" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+    </row>
+    <row r="52" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+    </row>
+    <row r="53" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+    </row>
+    <row r="54" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+    </row>
+    <row r="55" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+    </row>
+    <row r="56" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I56" s="3"/>
+      <c r="J56" s="3"/>
+    </row>
+    <row r="57" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+    </row>
+    <row r="58" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+    </row>
+    <row r="59" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
+    </row>
+    <row r="60" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+    </row>
+    <row r="61" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I61" s="3"/>
+      <c r="J61" s="3"/>
+    </row>
+    <row r="62" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I62" s="3"/>
+      <c r="J62" s="3"/>
+    </row>
+    <row r="63" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I63" s="3"/>
+      <c r="J63" s="3"/>
+    </row>
+    <row r="64" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I64" s="3"/>
+      <c r="J64" s="3"/>
+    </row>
+    <row r="65" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I65" s="3"/>
+      <c r="J65" s="3"/>
+    </row>
+    <row r="66" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I66" s="3"/>
+      <c r="J66" s="3"/>
+    </row>
+    <row r="67" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I67" s="3"/>
+      <c r="J67" s="3"/>
+    </row>
+    <row r="68" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I68" s="3"/>
+      <c r="J68" s="3"/>
+    </row>
+    <row r="69" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+    </row>
+    <row r="70" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I70" s="3"/>
+      <c r="J70" s="3"/>
+    </row>
+    <row r="71" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I71" s="3"/>
+      <c r="J71" s="3"/>
+    </row>
+    <row r="72" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I72" s="3"/>
+      <c r="J72" s="3"/>
+    </row>
+    <row r="73" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+    </row>
+    <row r="74" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I74" s="3"/>
+      <c r="J74" s="3"/>
+    </row>
+    <row r="75" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I75" s="3"/>
+      <c r="J75" s="3"/>
+    </row>
+    <row r="76" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+    </row>
+    <row r="77" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I77" s="3"/>
+      <c r="J77" s="3"/>
+    </row>
+    <row r="78" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
+    </row>
+    <row r="79" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I79" s="3"/>
+      <c r="J79" s="3"/>
+    </row>
+    <row r="80" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I80" s="3"/>
+      <c r="J80" s="3"/>
+    </row>
+    <row r="81" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I81" s="3"/>
+      <c r="J81" s="3"/>
+    </row>
+    <row r="82" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I82" s="3"/>
+      <c r="J82" s="3"/>
+    </row>
+    <row r="83" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I83" s="3"/>
+      <c r="J83" s="3"/>
+    </row>
+    <row r="84" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I84" s="3"/>
+      <c r="J84" s="3"/>
+    </row>
+    <row r="85" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I85" s="3"/>
+      <c r="J85" s="3"/>
+    </row>
+    <row r="86" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I86" s="3"/>
+      <c r="J86" s="3"/>
+    </row>
+    <row r="87" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I87" s="3"/>
+      <c r="J87" s="3"/>
+    </row>
+    <row r="88" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I88" s="3"/>
+      <c r="J88" s="3"/>
+    </row>
+    <row r="89" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I89" s="3"/>
+      <c r="J89" s="3"/>
+    </row>
+    <row r="90" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I90" s="3"/>
+      <c r="J90" s="3"/>
+    </row>
+    <row r="91" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I91" s="3"/>
+      <c r="J91" s="3"/>
+    </row>
+    <row r="92" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I92" s="3"/>
+      <c r="J92" s="3"/>
+    </row>
+    <row r="93" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I93" s="3"/>
+      <c r="J93" s="3"/>
+    </row>
+    <row r="94" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I94" s="3"/>
+      <c r="J94" s="3"/>
+    </row>
+    <row r="95" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I95" s="3"/>
+      <c r="J95" s="3"/>
+    </row>
+    <row r="96" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I96" s="3"/>
+      <c r="J96" s="3"/>
+    </row>
+    <row r="97" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I97" s="3"/>
+      <c r="J97" s="3"/>
+    </row>
+    <row r="98" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I98" s="3"/>
+      <c r="J98" s="3"/>
+    </row>
+    <row r="99" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I99" s="3"/>
+      <c r="J99" s="3"/>
+    </row>
+    <row r="100" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I100" s="3"/>
+      <c r="J100" s="3"/>
+    </row>
+    <row r="101" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I101" s="3"/>
+      <c r="J101" s="3"/>
+    </row>
+    <row r="102" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I102" s="3"/>
+      <c r="J102" s="3"/>
+    </row>
+    <row r="103" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I103" s="3"/>
+      <c r="J103" s="3"/>
+    </row>
+    <row r="104" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I104" s="3"/>
+      <c r="J104" s="3"/>
+    </row>
+    <row r="105" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I105" s="3"/>
+      <c r="J105" s="3"/>
+    </row>
+    <row r="106" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I106" s="3"/>
+      <c r="J106" s="3"/>
+    </row>
+    <row r="107" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I107" s="3"/>
+      <c r="J107" s="3"/>
+    </row>
+    <row r="108" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I108" s="3"/>
+      <c r="J108" s="3"/>
+    </row>
+    <row r="109" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I109" s="3"/>
+      <c r="J109" s="3"/>
+    </row>
+    <row r="110" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I110" s="3"/>
+      <c r="J110" s="3"/>
+    </row>
+    <row r="111" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I111" s="3"/>
+      <c r="J111" s="3"/>
+    </row>
+    <row r="112" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I112" s="3"/>
+      <c r="J112" s="3"/>
+    </row>
+    <row r="113" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I113" s="3"/>
+      <c r="J113" s="3"/>
+    </row>
+    <row r="114" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I114" s="3"/>
+      <c r="J114" s="3"/>
+    </row>
+    <row r="115" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I115" s="3"/>
+      <c r="J115" s="3"/>
+    </row>
+    <row r="116" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I116" s="3"/>
+      <c r="J116" s="3"/>
+    </row>
+    <row r="117" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I117" s="3"/>
+      <c r="J117" s="3"/>
+    </row>
+    <row r="118" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I118" s="3"/>
+      <c r="J118" s="3"/>
+    </row>
+    <row r="119" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I119" s="3"/>
+      <c r="J119" s="3"/>
+    </row>
+    <row r="120" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I120" s="3"/>
+      <c r="J120" s="3"/>
+    </row>
+    <row r="121" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I121" s="3"/>
+      <c r="J121" s="3"/>
+    </row>
+    <row r="122" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I122" s="3"/>
+      <c r="J122" s="3"/>
+    </row>
+    <row r="123" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I123" s="3"/>
+      <c r="J123" s="3"/>
+    </row>
+    <row r="124" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I124" s="3"/>
+      <c r="J124" s="3"/>
+    </row>
+    <row r="125" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I125" s="3"/>
+      <c r="J125" s="3"/>
+    </row>
+    <row r="126" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I126" s="3"/>
+      <c r="J126" s="3"/>
+    </row>
+    <row r="127" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I127" s="3"/>
+      <c r="J127" s="3"/>
+    </row>
+    <row r="128" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I128" s="3"/>
+      <c r="J128" s="3"/>
+    </row>
+    <row r="129" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I129" s="3"/>
+      <c r="J129" s="3"/>
+    </row>
+    <row r="130" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I130" s="3"/>
+      <c r="J130" s="3"/>
+    </row>
+    <row r="131" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I131" s="3"/>
+      <c r="J131" s="3"/>
+    </row>
+    <row r="132" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I132" s="3"/>
+      <c r="J132" s="3"/>
+    </row>
+    <row r="133" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I133" s="3"/>
+      <c r="J133" s="3"/>
+    </row>
+    <row r="134" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I134" s="3"/>
+      <c r="J134" s="3"/>
+    </row>
+    <row r="135" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I135" s="3"/>
+      <c r="J135" s="3"/>
+    </row>
+    <row r="136" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I136" s="3"/>
+      <c r="J136" s="3"/>
+    </row>
+    <row r="137" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I137" s="3"/>
+      <c r="J137" s="3"/>
+    </row>
+    <row r="138" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I138" s="3"/>
+      <c r="J138" s="3"/>
+    </row>
+    <row r="139" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I139" s="3"/>
+      <c r="J139" s="3"/>
+    </row>
+    <row r="140" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I140" s="3"/>
+      <c r="J140" s="3"/>
+    </row>
+    <row r="141" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I141" s="3"/>
+      <c r="J141" s="3"/>
+    </row>
+    <row r="142" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I142" s="3"/>
+      <c r="J142" s="3"/>
+    </row>
+    <row r="143" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I143" s="3"/>
+      <c r="J143" s="3"/>
+    </row>
+    <row r="144" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I144" s="3"/>
+      <c r="J144" s="3"/>
+    </row>
+    <row r="145" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I145" s="3"/>
+      <c r="J145" s="3"/>
+    </row>
+    <row r="146" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I146" s="3"/>
+      <c r="J146" s="3"/>
+    </row>
+    <row r="147" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I147" s="3"/>
+      <c r="J147" s="3"/>
+    </row>
+    <row r="148" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I148" s="3"/>
+      <c r="J148" s="3"/>
+    </row>
+    <row r="149" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I149" s="3"/>
+      <c r="J149" s="3"/>
+    </row>
+    <row r="150" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I150" s="3"/>
+      <c r="J150" s="3"/>
+    </row>
+    <row r="151" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I151" s="3"/>
+      <c r="J151" s="3"/>
+    </row>
+    <row r="152" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I152" s="3"/>
+      <c r="J152" s="3"/>
+    </row>
+    <row r="153" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I153" s="3"/>
+      <c r="J153" s="3"/>
+    </row>
+    <row r="154" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I154" s="3"/>
+      <c r="J154" s="3"/>
+    </row>
+    <row r="155" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I155" s="3"/>
+      <c r="J155" s="3"/>
+    </row>
+    <row r="156" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I156" s="3"/>
+      <c r="J156" s="3"/>
+    </row>
+    <row r="157" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I157" s="3"/>
+      <c r="J157" s="3"/>
+    </row>
+    <row r="158" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I158" s="3"/>
+      <c r="J158" s="3"/>
+    </row>
+    <row r="159" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I159" s="3"/>
+      <c r="J159" s="3"/>
+    </row>
+    <row r="160" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I160" s="3"/>
+      <c r="J160" s="3"/>
+    </row>
+    <row r="161" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I161" s="3"/>
+      <c r="J161" s="3"/>
+    </row>
+    <row r="162" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I162" s="3"/>
+      <c r="J162" s="3"/>
+    </row>
+    <row r="163" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I163" s="3"/>
+      <c r="J163" s="3"/>
+    </row>
+    <row r="164" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I164" s="3"/>
+      <c r="J164" s="3"/>
+    </row>
+    <row r="165" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I165" s="3"/>
+      <c r="J165" s="3"/>
+    </row>
+    <row r="166" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I166" s="3"/>
+      <c r="J166" s="3"/>
+    </row>
+    <row r="167" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I167" s="3"/>
+      <c r="J167" s="3"/>
+    </row>
+    <row r="168" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I168" s="3"/>
+      <c r="J168" s="3"/>
+    </row>
+    <row r="169" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I169" s="3"/>
+      <c r="J169" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>